<commit_message>
update listening 22_12 1-3
</commit_message>
<xml_diff>
--- a/LISTEN/Script/22_12/22_12.xlsx
+++ b/LISTEN/Script/22_12/22_12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\LISTEN\Script\22_12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89271D7C-2E6A-4334-9002-8CAB540BDBE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A1D1E6A-E6F0-4701-B38F-7E9E933BEF1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17895" yWindow="10230" windowWidth="26130" windowHeight="9255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14820" yWindow="4275" windowWidth="23580" windowHeight="9255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1番" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="156">
   <si>
     <t>Fre</t>
   </si>
@@ -429,6 +429,218 @@
   </si>
   <si>
     <t>上着</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>企画書</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>きかくしょ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>抑える</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>おさえる</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>抑制</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>甘さ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>あまさ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>甜度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>大人</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>おとな</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>箱</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>はこ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>盒子</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>高級感</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>こうきゅうかん</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>出す</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>だす</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>拿出、营造</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>狙い</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ねらい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目标、意图</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>販売</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>はんばい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>価格</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>かかく</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>設定</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>せってい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>〜だと</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>假定条件</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>店の棚</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>消費者</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>しょうひしゃ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目に止まる</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>めにとまる</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>注意到</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目立つ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>めだつ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>显眼</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>〜たりする</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>做……啦……啦</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>不完全列举</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>調整</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ちょうせい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>指摘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>してき</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>指出</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>修正</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>しゅうせい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>今のように</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>就像现在这样</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>十分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>じゅうぶん</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>みせのたな</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -759,7 +971,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -1305,6 +1517,286 @@
       </c>
       <c r="C44" s="2" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A45" s="1">
+        <v>0</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A46" s="1">
+        <v>0</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A47" s="1">
+        <v>0</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A48" s="1">
+        <v>0</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A49" s="1">
+        <v>0</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A50" s="1">
+        <v>0</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A51" s="1">
+        <v>0</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A52" s="1">
+        <v>0</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A53" s="1">
+        <v>0</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A54" s="1">
+        <v>0</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A55" s="1">
+        <v>0</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A56" s="1">
+        <v>0</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A57" s="1">
+        <v>0</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A58" s="1">
+        <v>0</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A59" s="1">
+        <v>0</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A60" s="1">
+        <v>0</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A61" s="1">
+        <v>0</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A62" s="1">
+        <v>0</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A63" s="1">
+        <v>0</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A64" s="1">
+        <v>0</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A65" s="1">
+        <v>0</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A66" s="1">
+        <v>0</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A67" s="1">
+        <v>0</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update listening 1-4 and 1-5
</commit_message>
<xml_diff>
--- a/LISTEN/Script/22_12/22_12.xlsx
+++ b/LISTEN/Script/22_12/22_12.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\LISTEN\Script\22_12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6B6CBE6-DEDD-4ACC-B098-FDB975FEC1DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46E3CEC-D4D5-48AB-B37E-48790D0462DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14820" yWindow="4275" windowWidth="23580" windowHeight="9255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="264">
   <si>
     <t>Fre</t>
   </si>
@@ -641,6 +641,437 @@
   </si>
   <si>
     <t>みせのたな</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>確か</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>たしか</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>好像是…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>金魚</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>きんぎょ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>飼ってる</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>かってる</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"飼っている"的口语</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>汚れちゃう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>よごれちゃう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"汚れてしまう"口语</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>しなきゃならない</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>必须…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"しなければならない"口语</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>水</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>みず</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>貝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>かい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>螺贝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2ヶ月前</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>にかげつまえ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>餌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>えさ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>饲料</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>りょう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日当</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ひあ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日照；阳光照射</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>影響</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>えいきょう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>〜通りに</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>とおりに</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>按照…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>玄関</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>げんかん</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>〜ずに</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>不…就…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>少ない</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>すくない</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>少</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>〜はいいとして</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>…暂且不论</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>中山</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>なかやま</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>新製品</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>しんせいひん</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>せんたくき</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>洗濯機</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>つける</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>附着在…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>マニュアルの案</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>说明书的草案</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>詳細な</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>しょうさいな</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>取扱</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>とりあつかい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>操作；使用</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>説明書</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>せつめいしょ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>簡単な</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>かんたんな</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>簡易</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>かんい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>印刷物</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>いんさつぶつ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>使い方</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>つかいかた</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>問題</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>もんだい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>文字</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>もじ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>絵</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>え</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>图片</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>シンプル</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>简单；简洁</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>簡潔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>かんけつ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>简洁；简明；扼要</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>動画</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>どうが</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>视频；动画</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>洗剤</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>せんざい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>洗涤剂</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>あんな</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>那样的；那种的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>余計な</t>
+  </si>
+  <si>
+    <t>よけいな</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多余的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>省く</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>はぶく</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>省略</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>字幕</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>じまく</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>複数</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ふくすう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多个</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>言語</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>げんご</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>语言</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>対応</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>たいおう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>对应</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ニーズ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>需求</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -971,13 +1402,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D111"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="11.25" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.25" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.75" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.125" style="1" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -1766,7 +2197,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A65" s="1">
         <v>0</v>
       </c>
@@ -1777,7 +2208,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A66" s="1">
         <v>0</v>
       </c>
@@ -1788,7 +2219,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A67" s="1">
         <v>0</v>
       </c>
@@ -1797,6 +2228,550 @@
       </c>
       <c r="C67" s="2" t="s">
         <v>154</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A68" s="1">
+        <v>0</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A69" s="1">
+        <v>0</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A70" s="1">
+        <v>0</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A71" s="1">
+        <v>0</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A72" s="1">
+        <v>0</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A73" s="1">
+        <v>0</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A74" s="1">
+        <v>0</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A75" s="1">
+        <v>0</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A76" s="1">
+        <v>0</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A77" s="1">
+        <v>0</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A78" s="1">
+        <v>0</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A79" s="1">
+        <v>0</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A80" s="1">
+        <v>0</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A81" s="1">
+        <v>0</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A82" s="1">
+        <v>0</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A83" s="1">
+        <v>0</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A84" s="1">
+        <v>0</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A85" s="1">
+        <v>0</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A86" s="1">
+        <v>0</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A87" s="1">
+        <v>0</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A88" s="1">
+        <v>0</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A89" s="1">
+        <v>0</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A90" s="1">
+        <v>0</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A91" s="1">
+        <v>0</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A92" s="1">
+        <v>0</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A93" s="1">
+        <v>0</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A94" s="1">
+        <v>0</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A95" s="1">
+        <v>0</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A96" s="1">
+        <v>0</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A97" s="1">
+        <v>0</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A98" s="1">
+        <v>0</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A99" s="1">
+        <v>0</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A100" s="1">
+        <v>0</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A101" s="1">
+        <v>0</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A102" s="1">
+        <v>0</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A103" s="1">
+        <v>0</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A104" s="1">
+        <v>0</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A105" s="1">
+        <v>0</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A106" s="1">
+        <v>0</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A107" s="1">
+        <v>0</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A108" s="1">
+        <v>0</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A109" s="1">
+        <v>0</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A110" s="1">
+        <v>0</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A111" s="1">
+        <v>0</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update 22_12 listen 1-4 & 1-5
</commit_message>
<xml_diff>
--- a/LISTEN/Script/22_12/22_12.xlsx
+++ b/LISTEN/Script/22_12/22_12.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\LISTEN\Script\22_12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D0E5FB-55FD-4E9B-8246-10994EDAE3FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359E21C1-9FA8-4191-94F1-9608AC31DD50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14820" yWindow="4275" windowWidth="23580" windowHeight="9255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="265">
   <si>
     <t>Fre</t>
   </si>
@@ -929,10 +929,6 @@
   </si>
   <si>
     <t>文字</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>もじ</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1963,10 +1959,10 @@
         <v>0</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>264</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.15">
@@ -2620,7 +2616,7 @@
         <v>227</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>228</v>
+        <v>24</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.15">
@@ -2628,13 +2624,13 @@
         <v>0</v>
       </c>
       <c r="B100" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C100" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="C100" s="2" t="s">
+      <c r="D100" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="D100" s="2" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.15">
@@ -2642,10 +2638,10 @@
         <v>0</v>
       </c>
       <c r="B101" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C101" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.15">
@@ -2653,13 +2649,13 @@
         <v>0</v>
       </c>
       <c r="B102" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C102" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C102" s="2" t="s">
+      <c r="D102" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.15">
@@ -2667,13 +2663,13 @@
         <v>0</v>
       </c>
       <c r="B103" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="C103" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="C103" s="2" t="s">
+      <c r="D103" s="2" t="s">
         <v>238</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.15">
@@ -2681,13 +2677,13 @@
         <v>0</v>
       </c>
       <c r="B104" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C104" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="C104" s="2" t="s">
+      <c r="D104" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.15">
@@ -2695,10 +2691,10 @@
         <v>0</v>
       </c>
       <c r="B105" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C105" s="2" t="s">
         <v>243</v>
-      </c>
-      <c r="C105" s="2" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.15">
@@ -2706,13 +2702,13 @@
         <v>0</v>
       </c>
       <c r="B106" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C106" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="C106" s="2" t="s">
+      <c r="D106" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.15">
@@ -2720,13 +2716,13 @@
         <v>0</v>
       </c>
       <c r="B107" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C107" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="C107" s="2" t="s">
+      <c r="D107" s="2" t="s">
         <v>249</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.15">
@@ -2734,10 +2730,10 @@
         <v>0</v>
       </c>
       <c r="B108" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C108" s="2" t="s">
         <v>251</v>
-      </c>
-      <c r="C108" s="2" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.15">
@@ -2745,13 +2741,13 @@
         <v>0</v>
       </c>
       <c r="B109" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C109" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="C109" s="2" t="s">
+      <c r="D109" s="2" t="s">
         <v>254</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.15">
@@ -2759,13 +2755,13 @@
         <v>0</v>
       </c>
       <c r="B110" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C110" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="C110" s="2" t="s">
+      <c r="D110" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.15">
@@ -2773,13 +2769,13 @@
         <v>0</v>
       </c>
       <c r="B111" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C111" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="C111" s="2" t="s">
+      <c r="D111" s="2" t="s">
         <v>260</v>
-      </c>
-      <c r="D111" s="2" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.15">
@@ -2787,10 +2783,10 @@
         <v>0</v>
       </c>
       <c r="B112" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C112" s="2" t="s">
         <v>262</v>
-      </c>
-      <c r="C112" s="2" t="s">
-        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>